<commit_message>
Schedule twice daily (10:00 AM & 9:00 PM IST) and commit latest outputs
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-05.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-05.xlsx
@@ -42,7 +42,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
         <bgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -111,7 +117,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -479,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -549,17 +558,262 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>atomic energy</t>
+          <t>atomic energy, uranium</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Aligined with General Studies 3 topics: atomic energy</t>
+          <t>Aligned with General Studies 3 topics: atomic energy, uranium</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2318970</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>India and Japan Launch Operational Manual for the Joint Crediting Mechanism</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>climate change</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319373</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>CAQM intensifies field-level monitoring with deployment of Flying Squads to prevent paddy stubble burning incidents in Punjab and Haryana</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>climate change, caqm</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319355</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Indian-born Cheetah gives birth to 5 Healthy Cubs at Kuno National Park; India’s Cheetah Population reaches 60</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>climate change, national park</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change, national park</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319097</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Appointment of Additional Judge of the Delhi High Court</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>high court</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: high court</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319338</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Appointment of Chief Justices of High Courts as Judges of the Supreme Court of India</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>supreme court</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: supreme court</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319337</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of New and Renewable Energy</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Union Minister Shri Pralhad Joshi to Inaugurate Windergy India 2026 in Chennai</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>renewable energy</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: renewable energy</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319302</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Road Transport &amp; Highways</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Union Minister Shri Nitin Gadkari Inaugurates Chintan Shivir 2026, Sets Agenda for Future-Ready Highway Infrastructure</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: infrastructure</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319085</t>
         </is>
       </c>
     </row>
@@ -574,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -586,32 +840,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>S.No.</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Classification</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Paper</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Ministry</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Headline</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>PIB URL</t>
         </is>
@@ -623,27 +877,1197 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>President's Secretariat</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PRESIDENT OF INDIA HOSTS PRESIDENT OF THE SWISS CONFEDERATION</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319423</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>President's Secretariat</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PRESIDENT OF INDIA TO VISIT HIMACHAL PRADESH FROM OCTOBER 6 TO 8</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319361</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>List of Outcomes: State Visit of President of the Swiss Confederation to India</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319109</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>English Translation of Press statement by the Prime Minister during the Joint Press Statement with the President of Switzerland</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319086</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Prime Minister shares Sanskrit Subhashitam highlighting the qualities of a noble-hearted person</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2318982</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AYUSH</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Integrated Ayurveda-Yoga Approach Shows Encouraging Results in Management of Bedwetting Among Children: ITRA Study</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319152</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Relevant (UPSC)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>GS-3</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Department of Atomic Energy</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>UCIL Celebrates Diamond Jubilee Year, Marks Six Decades of India’s Uranium Mining and Processing Capability</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2318970</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ministry of Coal</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>From Coal Availability to Energy Security: CIL Strengthens Coal Supply and Distribution to Power Sector</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319084</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ministry of Communications</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Union Minister of Communications Shri Jyotiraditya M. Scindia Reviews Final Preparations for IMC 2026 at Yashobhoomi</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319395</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Ministry of Communications</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>“The Indian Telecom Services Yearly Performance Indicators” for the year 2025-26</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319321</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ministry of Communications</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sanchar Saathi portal crosses 30 crore visits as citizens turn Cyber Warriors against telecom fraud</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319087</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ministry of Corporate Affairs</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>IICA observed 3rd IICA CSR Day on Gandhi Jayanti with a Special Address by the DG &amp; CEO to Participants of the IICA Certified CSR Professional Programme ahead of NCCSR 2026</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319348</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Raksha Mantri Shri Rajnath Singh Underscores India’s Rising Maritime Power, Indigenous Naval Capability and Strategic Strength at Barakhana in Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319425</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Raksha Mantri to mark delivery of 2,000th aero-engine at HAL Koraput tomorrow</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319187</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Raksha Mantri Shri Rajnath Singh to Launch First Fleet Support Ship (FSS-1), Lay Keel of FSS-5 and Inaugurate Upgraded Slipway-4 &amp; 300-Tonne Goliath Crane at Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319156</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>INDIA-UAE JOINT MILITARY EXERCISE MOUNTAIN GUARDIAN 2026 COMMENCES IN UTTARAKHAND</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319135</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>India and Japan Launch Operational Manual for the Joint Crediting Mechanism</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319373</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CAQM intensifies field-level monitoring with deployment of Flying Squads to prevent paddy stubble burning incidents in Punjab and Haryana</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319355</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Indian-born Cheetah gives birth to 5 Healthy Cubs at Kuno National Park; India’s Cheetah Population reaches 60</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319097</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ministry of Housing &amp; Urban Affairs</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MoHUA celebrates World Habitat Day 2026 with focus on advancing affordable, resilient and Inclusive housing</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319398</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Appointment of Additional Judge of the Delhi High Court</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319338</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Appointment of Chief Justices of High Courts as Judges of the Supreme Court of India</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319337</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Ministry of New and Renewable Energy</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Union Minister Shri Pralhad Joshi to Inaugurate Windergy India 2026 in Chennai</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319302</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Ministries/Departments of Government of India geared up for implementation phase of Special Campaign 6 from 2nd-31st October, 2026</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319335</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Dr. Jitendra Singh Reiterates Commitment to Ease of Life for Pensioners; Calls for Wider Adoption of Digital Pension Services</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319228</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Dr. Jitendra Singh Reviews Progress of Special Campaign 6 at DARPG Office, Sardar Patel Bhawan, New Delhi</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319204</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Ministry of Road Transport &amp; Highways</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Union Minister Shri Nitin Gadkari Inaugurates Chintan Shivir 2026, Sets Agenda for Future-Ready Highway Infrastructure</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319085</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Ministry of Science &amp; Technology</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>“Swachhata Hi Sewa-2026” campaign</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319076</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Ministry of Science &amp; Technology</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>TDB-DST signs agreement with BigEndian Semiconductors for ₹130 crore RDI support to develop indigenous AI Vision SoC</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319038</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Ministry of Ports, Shipping and Waterways</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Dibrugarh Sends First International Cargo from Bogibeel to Bangladesh Since Independence</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319146</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2nd Prof. (Dr.) N. R. Madhava Menon Memorial Lecture Held at Dr. Ambedkar International Centre</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319413</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>From Unemployment to Self-Reliance</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319229</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>From Financial Constraints to Academic Aspirations</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319191</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>From Waste Picker to Entrepreneur</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319117</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Ministry of Statistics &amp; Programme Implementation</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>National Household Travel Survey July, 2025 – June, 2026</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319180</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Ministry of Textiles</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Ministry of Textiles Organises Swachhta and Cleanliness Activities on Gandhi Jayanti under Special Campaign 6</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319367</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Ministry of Youth Affairs and Sports</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Department of Sports to participate in Special Campaign 6.0 to enhance cleanliness and resolve pending matters</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319171</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>PIB Backgrounder</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Saving Time, Shortening Journeys</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319049</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>National Human Rights Commission</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>NHRC, India to hold 'Open Hearing and Camp Sitting' at Patna to hear cases of alleged human rights violations in Bihar on 7th-8th October 2026</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319221</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ministry of Chemicals and Fertilizers - Department of Chemicals and Petrochemicals</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Union Minister of State for Chemicals and Fertilizers Anupriya Patel Launches 14th Edition of India Chem 2026</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319421</t>
         </is>
       </c>
     </row>

</xml_diff>